<commit_message>
revisions protocol and imports' files
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations /ClimOO Imports.xlsx
+++ b/ClimOO material/materials for implementations /ClimOO Imports.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD5731F9-B586-5C4B-996F-9A987338CC11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A265FE2-2DDF-824F-888B-B84FE1B7FB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16420" activeTab="1" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
   </bookViews>
   <sheets>
     <sheet name="Ontologies reused" sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="355">
   <si>
     <t>Agri-Food Experiment Ontology</t>
   </si>
@@ -88,9 +88,6 @@
     <t>Climate Crisis Management Ontology</t>
   </si>
   <si>
-    <t>10.5281/zenodo.1243535</t>
-  </si>
-  <si>
     <t>Ecosystem Ontology</t>
   </si>
   <si>
@@ -295,30 +292,18 @@
     <t>CHIRO</t>
   </si>
   <si>
-    <t>The Ecosystem Ontology (ECSO)</t>
-  </si>
-  <si>
     <t>SnowTerm Thesaurus </t>
   </si>
   <si>
     <t>SWEET</t>
   </si>
   <si>
-    <t>Ontology of bioscientific data analysis and data management (EDAM)</t>
-  </si>
-  <si>
-    <t>Evidence and Conclusion Ontology (ECO)</t>
-  </si>
-  <si>
     <t>National Agricultural Library Thesaurus (NALT)</t>
   </si>
   <si>
     <t>maybe</t>
   </si>
   <si>
-    <t>AgrOntology (AGRONTOLOGY)</t>
-  </si>
-  <si>
     <t>Common Ontology of Value and Risk</t>
   </si>
   <si>
@@ -358,9 +343,6 @@
     <t>Weathering Ontology</t>
   </si>
   <si>
-    <t>Environmental Thesaurus (ENVTHES)</t>
-  </si>
-  <si>
     <t>Sensor, Observation, Sample, and Actuator Ontology (SOSA)</t>
   </si>
   <si>
@@ -586,9 +568,6 @@
     <t>CPMETA</t>
   </si>
   <si>
-    <t>√https://github.com/ICOS-Carbon-Portal/meta/blob/master/src/main/resources/owl/cpmeta.owl</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ontology of Experimental Events </t>
   </si>
   <si>
@@ -1010,6 +989,120 @@
   </si>
   <si>
     <t>Process and Observation Ontology</t>
+  </si>
+  <si>
+    <t>CA Ontology</t>
+  </si>
+  <si>
+    <t>Climate Analysis Ontology</t>
+  </si>
+  <si>
+    <t>https://github.com/futaoo/codespaceRepo</t>
+  </si>
+  <si>
+    <t>Climate and Forecast (CF) vocabulary</t>
+  </si>
+  <si>
+    <t>CF Vocabulary</t>
+  </si>
+  <si>
+    <t>HERACLES Ontology</t>
+  </si>
+  <si>
+    <t>HEritage Resilience Against CLimate Events on Site Ontology</t>
+  </si>
+  <si>
+    <t>https://github.com/FraunhoferIOSB/HERACLES</t>
+  </si>
+  <si>
+    <t>GCIS Ontology</t>
+  </si>
+  <si>
+    <t>Global Change Information System Ontology</t>
+  </si>
+  <si>
+    <t>https://github.com/USGCRP/gcis-ontology</t>
+  </si>
+  <si>
+    <t>climate smart agriculture ontology</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> OntoCSA</t>
+  </si>
+  <si>
+    <t>https://github.com/sfpileggi/CCTL-Ontology</t>
+  </si>
+  <si>
+    <t>CCTL Ontology</t>
+  </si>
+  <si>
+    <t>Climate Change Time-Line ontology</t>
+  </si>
+  <si>
+    <t>PPCinIM ontology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/psapel/PPCinIM </t>
+  </si>
+  <si>
+    <t>An ontology for production planning and control in njection molding</t>
+  </si>
+  <si>
+    <t>OntoEndo</t>
+  </si>
+  <si>
+    <t>Core Ontology of Endogenous Knowledge on Agricultural Techniques</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1007/978-3-031-34896-9_12</t>
+  </si>
+  <si>
+    <t>Repository/Homepage/Reference</t>
+  </si>
+  <si>
+    <t>Climate Change Ontology</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1007/978-3-030-71187-0_104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/ICOS-Carbon-Portal </t>
+  </si>
+  <si>
+    <t>Environmental Thesaurus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ontology of bioscientific data analysis and data management </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Ecosystem Ontology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence and Conclusion Ontology </t>
+  </si>
+  <si>
+    <t>AgrOntology</t>
+  </si>
+  <si>
+    <t>DDR Ontology</t>
+  </si>
+  <si>
+    <t>Domain Ontology for Learning Resources on Disaster Risk Reduction</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.procs.2024.09.319</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://bigdata.cgiar.org/resources/agronomy-ontology/ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.4018/IJAEIS.292476 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.w3.org/2005/Incubator/ssn/ssnx/cf/cf-property </t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.5281/zenodo.1243535 </t>
   </si>
 </sst>
 </file>
@@ -1204,7 +1297,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1215,9 +1308,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1244,9 +1334,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1302,7 +1389,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1659,7 +1754,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2C20A25-ACC7-684D-AF97-19E64433B7DC}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
@@ -1668,256 +1763,259 @@
     <col min="4" max="4" width="14.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="35" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="35" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="35" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="35" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="B2" s="23" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>68</v>
-      </c>
-      <c r="D2" s="23" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="23" t="s">
+      <c r="C3" s="28" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="D3" s="21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="30" t="s">
-        <v>70</v>
-      </c>
-      <c r="D3" s="23" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
+      <c r="C4" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="D4" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="21" t="s">
+        <v>286</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>285</v>
+      </c>
+      <c r="C6" s="28" t="s">
+        <v>287</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="21" t="s">
+        <v>282</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>283</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>284</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="21" t="s">
+        <v>306</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>292</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>298</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="21" t="s">
+        <v>305</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>293</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>299</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>295</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="21" t="s">
+        <v>302</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>296</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="21" t="s">
+        <v>303</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>294</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>301</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="21" t="s">
+        <v>304</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>300</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="21" t="s">
+        <v>307</v>
+      </c>
+      <c r="B14" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C14" s="21" t="s">
+        <v>297</v>
+      </c>
+      <c r="D14" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="D4" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="30" t="s">
-        <v>77</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="23" t="s">
-        <v>293</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>292</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>294</v>
-      </c>
-      <c r="D6" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="23" t="s">
-        <v>289</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>290</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>291</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="23" t="s">
+    </row>
+    <row r="15" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="24" t="s">
+        <v>251</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>250</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>249</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="34" t="s">
+        <v>311</v>
+      </c>
+      <c r="B16" s="34" t="s">
+        <v>312</v>
+      </c>
+      <c r="C16" s="35" t="s">
         <v>313</v>
       </c>
-      <c r="B8" s="23" t="s">
-        <v>299</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>305</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="23" t="s">
-        <v>312</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>300</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>306</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
-        <v>295</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>302</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="23" t="s">
-        <v>309</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>303</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="23" t="s">
-        <v>310</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>301</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>308</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="23" t="s">
-        <v>311</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>307</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="23" t="s">
-        <v>314</v>
-      </c>
-      <c r="B14" s="23" t="s">
+      <c r="D16" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="G16" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="21" t="s">
+        <v>165</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="21" t="s">
+        <v>277</v>
+      </c>
+      <c r="B18" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="23" t="s">
-        <v>304</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="26" t="s">
-        <v>258</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>257</v>
-      </c>
-      <c r="C15" s="25" t="s">
-        <v>256</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="36" t="s">
-        <v>318</v>
-      </c>
-      <c r="B16" s="36" t="s">
-        <v>319</v>
-      </c>
-      <c r="C16" s="37" t="s">
-        <v>320</v>
-      </c>
-      <c r="D16" s="36" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>170</v>
-      </c>
-      <c r="D17" s="36" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="39" t="s">
-        <v>284</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="30" t="s">
-        <v>283</v>
-      </c>
-      <c r="D18" s="36" t="s">
-        <v>74</v>
+      <c r="C18" s="28" t="s">
+        <v>276</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>73</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1932,6 +2030,8 @@
     <hyperlink ref="C16" r:id="rId6" xr:uid="{13BBB7FD-8082-2D42-9493-20D5AF29854A}"/>
     <hyperlink ref="C17" r:id="rId7" xr:uid="{D3895E0F-1B7A-1C47-B577-5C63E642DBE7}"/>
     <hyperlink ref="C18" r:id="rId8" xr:uid="{3B5A9A2C-530A-1043-94EC-CC59816CE215}"/>
+    <hyperlink ref="C6" r:id="rId9" xr:uid="{F3E73C96-B4DA-DF4F-9696-842581A6C68D}"/>
+    <hyperlink ref="C9" r:id="rId10" xr:uid="{E3D2B798-0F52-754A-B5EC-3ED2EAFAC7FF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -1940,72 +2040,72 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B475128C-F7EE-8540-83D5-7C0DBC4F277D}">
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="75.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="110.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="B1" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>339</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="6" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="25" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
-        <v>275</v>
-      </c>
-      <c r="B3" s="9" t="s">
+    </row>
+    <row r="3" spans="1:6" s="6" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="21" t="s">
+        <v>268</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="E3" s="32" t="s">
+        <v>308</v>
+      </c>
+      <c r="F3" s="29"/>
+    </row>
+    <row r="4" spans="1:6" s="6" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
+        <v>274</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C4" s="23" t="s">
         <v>273</v>
       </c>
-      <c r="C3" s="25" t="s">
-        <v>274</v>
-      </c>
-      <c r="E3" s="34" t="s">
-        <v>315</v>
-      </c>
-      <c r="F3" s="31"/>
-    </row>
-    <row r="4" spans="1:6" s="7" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
-        <v>281</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>280</v>
-      </c>
-      <c r="E4" s="32"/>
-      <c r="F4" s="33" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="E4" s="30"/>
+      <c r="F4" s="31" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>0</v>
       </c>
@@ -2013,120 +2113,120 @@
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="23" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="21" t="s">
+        <v>271</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="39" t="s">
+        <v>347</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>257</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="19" t="s">
+        <v>279</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="28" t="s">
         <v>278</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="C8" s="25" t="s">
-        <v>264</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
-        <v>286</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>285</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
       <c r="F9"/>
     </row>
-    <row r="10" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
-        <v>260</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="25" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C11" s="23" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="25" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="7" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="21" t="s">
-        <v>268</v>
-      </c>
-      <c r="B14" s="9" t="s">
+      <c r="C13" s="23" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="6" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="19" t="s">
+        <v>261</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>267</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C14" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>11</v>
@@ -2135,9 +2235,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>6</v>
@@ -2146,845 +2246,989 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="25" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="27" t="s">
-        <v>253</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C20" s="25" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="B21" s="9" t="s">
+      <c r="C18" s="23" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="8" t="s">
         <v>245</v>
       </c>
-      <c r="C21" s="25" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="B22" s="9" t="s">
+    </row>
+    <row r="20" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="C20" s="23" t="s">
         <v>247</v>
       </c>
-      <c r="C22" s="25" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="15" t="s">
+    </row>
+    <row r="21" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>239</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="39" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="39" t="s">
+        <v>174</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="C23" s="40" t="s">
+        <v>342</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="21" t="s">
+        <v>223</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="39" t="s">
+        <v>346</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" s="6" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A29" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="26" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="41" t="s">
+        <v>345</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="39" t="s">
+        <v>344</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="C32" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>181</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C24" s="25" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="25" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="C26" s="25" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="B27" s="9" t="s">
+    </row>
+    <row r="33" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="21" t="s">
+        <v>210</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="19" t="s">
+        <v>343</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="C35" s="23" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="B36" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="C27" s="25" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" s="7" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="A29" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C29" s="28" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" s="25" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="B31" s="4" t="s">
+      <c r="C36" s="23" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C37" s="23" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C31" s="25" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="C32" s="25" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="23" t="s">
-        <v>217</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="C33" s="25" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="B35" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="C35" s="25" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="21" t="s">
-        <v>224</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="C36" s="25" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="21" t="s">
-        <v>222</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="C37" s="25" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="16" t="s">
+      <c r="B38" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="C38" s="4" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="21" t="s">
-        <v>282</v>
-      </c>
-      <c r="B39" s="29" t="s">
-        <v>287</v>
-      </c>
-      <c r="C39" s="30" t="s">
-        <v>288</v>
+        <v>208</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="19" t="s">
+        <v>275</v>
+      </c>
+      <c r="B39" s="27" t="s">
+        <v>280</v>
+      </c>
+      <c r="C39" s="28" t="s">
+        <v>281</v>
       </c>
       <c r="D39"/>
       <c r="E39"/>
       <c r="F39"/>
     </row>
-    <row r="40" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>24</v>
-      </c>
       <c r="C40" s="4" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="B41" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="C41" s="25" t="s">
-        <v>210</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="23" t="s">
-        <v>211</v>
-      </c>
-      <c r="B42" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="C42" s="25" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="23" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C41" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="21" t="s">
         <v>204</v>
       </c>
-      <c r="B43" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="B44" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="C44" s="12" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="8" t="s">
+      <c r="B42" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C42" s="23" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="B43" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="C43" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="C45" s="9" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="23" t="s">
+    </row>
+    <row r="44" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="39" t="s">
+        <v>191</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C46" s="23" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C48" s="23" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="C49" s="23" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="B50" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="C50" s="23" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="C51" s="23" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="39" t="s">
+        <v>243</v>
+      </c>
+      <c r="B52" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="B46" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="C46" s="25" t="s">
+      <c r="B53" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C53" s="8" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="18" t="s">
+    <row r="54" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C54" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="B47" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="B48" s="9" t="s">
+    </row>
+    <row r="55" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="C55" s="23" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C56" s="23" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="B57" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="C57" s="23" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C58" s="23" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B59" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="39" t="s">
+        <v>160</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C60" s="23" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="C61" s="11" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="C62" s="23" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C63" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="C48" s="25" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="B49" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="C49" s="25" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="B50" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="C50" s="25" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="23" t="s">
-        <v>161</v>
-      </c>
-      <c r="B51" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="C51" s="25" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="8" t="s">
-        <v>250</v>
-      </c>
-      <c r="B52" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="C52" s="9" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="23" t="s">
+    </row>
+    <row r="64" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B65" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="C65" s="23" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="B66" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="C66" s="23" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B67" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="B53" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="C53" s="9" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="B54" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="C54" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="23" t="s">
-        <v>183</v>
-      </c>
-      <c r="B55" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="C55" s="25" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C56" s="25" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="17" t="s">
-        <v>123</v>
-      </c>
-      <c r="B57" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="C57" s="25" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="21" t="s">
-        <v>192</v>
-      </c>
-      <c r="B58" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="C58" s="25" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B59" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="C59" s="9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="B60" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="C60" s="25" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="23" t="s">
+      <c r="C67" s="23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="B61" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="C61" s="12" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="B62" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="C62" s="25" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C63" s="25" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B65" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="C65" s="25" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="14" t="s">
+      <c r="B68" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="C68" s="23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="B66" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="C66" s="25" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B67" s="22" t="s">
+      <c r="B69" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="C69" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="C67" s="25" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="C68" s="25" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="B69" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="C69" s="25" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="21" t="s">
-        <v>296</v>
-      </c>
-      <c r="B70" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="C70" s="30" t="s">
-        <v>201</v>
+    </row>
+    <row r="70" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="B70" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="C70" s="28" t="s">
+        <v>194</v>
       </c>
       <c r="D70"/>
       <c r="E70"/>
       <c r="F70"/>
     </row>
-    <row r="71" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="23" t="s">
-        <v>241</v>
-      </c>
-      <c r="B71" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="C71" s="25" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="21" t="s">
-        <v>239</v>
-      </c>
-      <c r="B72" s="26" t="s">
-        <v>238</v>
-      </c>
-      <c r="C72" s="25" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="B73" s="26" t="s">
-        <v>236</v>
-      </c>
-      <c r="C73" s="25" t="s">
+    <row r="71" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="21" t="s">
+        <v>234</v>
+      </c>
+      <c r="B71" s="8" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="21" t="s">
+      <c r="C71" s="23" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="B74" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="C74" s="25" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B72" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="C72" s="23" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="B73" s="24" t="s">
+        <v>229</v>
+      </c>
+      <c r="C73" s="23" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="C74" s="23" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C75" s="25" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="B76" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="C76" s="25" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="C75" s="23" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="39" t="s">
+        <v>166</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="C76" s="23" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B77" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B77" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C77" s="25" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" s="7" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="B78" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="C78" s="9" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="B79" s="9"/>
-      <c r="C79" s="9" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" s="7" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="16" t="s">
+      <c r="C77" s="23" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" s="6" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B78" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="B79" s="8"/>
+      <c r="C79" s="8" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" s="6" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="14" t="s">
         <v>15</v>
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="B81" s="12"/>
-      <c r="C81" s="13" t="s">
-        <v>244</v>
+        <v>354</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B81" s="11"/>
+      <c r="C81" s="12" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A82" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="B82" s="12"/>
-      <c r="C82" s="25" t="s">
-        <v>243</v>
-      </c>
-      <c r="D82" s="7"/>
-      <c r="E82" s="7"/>
-      <c r="F82" s="7"/>
+      <c r="A82" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="B82" s="11"/>
+      <c r="C82" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="D82" s="6"/>
+      <c r="E82" s="6"/>
+      <c r="F82" s="6"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="D83" s="7"/>
-      <c r="E83" s="7"/>
-      <c r="F83" s="7"/>
+        <v>194</v>
+      </c>
+      <c r="D83" s="6"/>
+      <c r="E83" s="6"/>
+      <c r="F83" s="6"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A84" s="16" t="s">
-        <v>26</v>
+      <c r="A84" s="14" t="s">
+        <v>25</v>
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D84" s="7"/>
-      <c r="E84" s="7"/>
-      <c r="F84" s="7"/>
+        <v>26</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E84" s="6"/>
+      <c r="F84" s="6"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A85" s="21" t="s">
+      <c r="A85" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="B85" s="11"/>
+      <c r="C85" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="D85" s="6"/>
+      <c r="E85" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F85" s="6"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A86" s="39" t="s">
+        <v>94</v>
+      </c>
+      <c r="B86" s="11"/>
+      <c r="C86" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="D86" s="6"/>
+      <c r="E86" s="6"/>
+      <c r="F86" s="6"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A87" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="B87" s="11"/>
+      <c r="C87" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E87" s="6"/>
+      <c r="F87" s="6"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A88" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="B88" s="11"/>
+      <c r="C88" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="D88" s="6"/>
+      <c r="E88" s="6"/>
+      <c r="F88" s="6"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A89" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="B85" s="12"/>
-      <c r="C85" s="25" t="s">
-        <v>194</v>
-      </c>
-      <c r="D85" s="7"/>
-      <c r="E85" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F85" s="7"/>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A86" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="B86" s="12"/>
-      <c r="C86" s="25" t="s">
-        <v>189</v>
-      </c>
-      <c r="D86" s="7"/>
-      <c r="E86" s="7"/>
-      <c r="F86" s="7"/>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A87" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="B87" s="12"/>
-      <c r="C87" s="25" t="s">
-        <v>188</v>
-      </c>
-      <c r="D87" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E87" s="7"/>
-      <c r="F87" s="7"/>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A88" s="23" t="s">
+      <c r="B89" s="11"/>
+      <c r="C89" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="D89" s="6"/>
+      <c r="E89" s="6"/>
+      <c r="F89" s="6"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A90" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="B88" s="12"/>
-      <c r="C88" s="25" t="s">
-        <v>176</v>
-      </c>
-      <c r="D88" s="7"/>
-      <c r="E88" s="7"/>
-      <c r="F88" s="7"/>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A89" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="B89" s="12"/>
-      <c r="C89" s="25" t="s">
-        <v>165</v>
-      </c>
-      <c r="D89" s="7"/>
-      <c r="E89" s="7"/>
-      <c r="F89" s="7"/>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A90" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="B90" s="12"/>
-      <c r="C90" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="D90" s="7"/>
-      <c r="E90" s="7"/>
-      <c r="F90" s="7"/>
+      <c r="B90" s="11"/>
+      <c r="C90" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="D90" s="6"/>
+      <c r="E90" s="6"/>
+      <c r="F90" s="6"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
+        <v>316</v>
+      </c>
+      <c r="B91" t="s">
+        <v>314</v>
+      </c>
+      <c r="C91" s="36" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>318</v>
+      </c>
+      <c r="B92" t="s">
+        <v>317</v>
+      </c>
+      <c r="C92" s="36" t="s">
+        <v>319</v>
+      </c>
+      <c r="D92" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>320</v>
+      </c>
+      <c r="B93" t="s">
+        <v>321</v>
+      </c>
+      <c r="C93" s="36" t="s">
+        <v>353</v>
+      </c>
+      <c r="D93" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
         <v>323</v>
       </c>
-      <c r="B91" t="s">
-        <v>321</v>
-      </c>
-      <c r="C91" s="38" t="s">
+      <c r="B94" t="s">
         <v>322</v>
+      </c>
+      <c r="C94" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A95" s="37" t="s">
+        <v>326</v>
+      </c>
+      <c r="B95" t="s">
+        <v>325</v>
+      </c>
+      <c r="C95" s="36" t="s">
+        <v>327</v>
+      </c>
+      <c r="D95" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A96" s="34" t="s">
+        <v>328</v>
+      </c>
+      <c r="B96" t="s">
+        <v>329</v>
+      </c>
+      <c r="C96" s="36" t="s">
+        <v>352</v>
+      </c>
+      <c r="D96" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>332</v>
+      </c>
+      <c r="B97" t="s">
+        <v>331</v>
+      </c>
+      <c r="C97" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A98" s="38" t="s">
+        <v>335</v>
+      </c>
+      <c r="B98" t="s">
+        <v>333</v>
+      </c>
+      <c r="C98" s="36" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>337</v>
+      </c>
+      <c r="B99" t="s">
+        <v>336</v>
+      </c>
+      <c r="C99" s="36" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>340</v>
+      </c>
+      <c r="C100" s="36" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A101" s="38" t="s">
+        <v>349</v>
+      </c>
+      <c r="B101" t="s">
+        <v>348</v>
+      </c>
+      <c r="C101" s="36" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>282</v>
+      </c>
+      <c r="B102" t="s">
+        <v>283</v>
+      </c>
+      <c r="C102" s="36" t="s">
+        <v>351</v>
       </c>
     </row>
   </sheetData>
@@ -2999,79 +3243,76 @@
     <hyperlink ref="C64" r:id="rId5" xr:uid="{C6F40C8D-7190-B740-B426-605371E8ECF8}"/>
     <hyperlink ref="C47" r:id="rId6" xr:uid="{A4D49E13-D104-8649-9EC7-2550F793CAD4}"/>
     <hyperlink ref="C54" r:id="rId7" xr:uid="{B787D633-212B-B248-9307-3E1160DF1616}"/>
-    <hyperlink ref="A30" r:id="rId8" display="https://ecoportal.lifewatch.eu/ontologies/ECSO" xr:uid="{489A4471-C877-F24D-930D-E81D9F374810}"/>
-    <hyperlink ref="A23" r:id="rId9" display="https://ecoportal.lifewatch.eu/ontologies/CPMETA" xr:uid="{F56D74CE-A25A-D945-B0FC-F5827574981B}"/>
-    <hyperlink ref="A32" r:id="rId10" display="https://biodivportal.gfbio.org/ontologies/EDAM" xr:uid="{05E273E9-A029-9643-A707-D384B4637DC0}"/>
-    <hyperlink ref="A60" r:id="rId11" display="https://biodivportal.gfbio.org/ontologies/QUDT" xr:uid="{9C2C2B49-4FA5-224C-8CDA-C2FF9E132E7B}"/>
-    <hyperlink ref="A27" r:id="rId12" display="https://biodivportal.gfbio.org/ontologies/ECO" xr:uid="{B297B450-7DF2-BE4D-92C9-78500CB10ED6}"/>
-    <hyperlink ref="A45" r:id="rId13" display="https://agroportal.lirmm.fr/ontologies/INRAETHES" xr:uid="{C71C31BE-87FF-0540-B26B-F6CEFAB9E223}"/>
-    <hyperlink ref="A76" r:id="rId14" display="https://agroportal.lirmm.fr/ontologies/TRANSFORMON" xr:uid="{7900C719-E36D-9F49-A23A-081FF403C10B}"/>
-    <hyperlink ref="A8" r:id="rId15" display="https://agroportal.lirmm.fr/ontologies/AGRONTOLOGY" xr:uid="{22EC63C0-9A81-6045-B4AD-452C2F098677}"/>
-    <hyperlink ref="A22" r:id="rId16" display="https://scs-ontouml.eemcs.utwente.nl/model/ef85708e-02ce-40b4-8fdb-57799201ee28" xr:uid="{A0736C9C-D991-7E40-966A-7E4DBD6E9F8B}"/>
-    <hyperlink ref="A86" r:id="rId17" display="https://scs-ontouml.eemcs.utwente.nl/model/87dea242-75d9-4b89-99f3-6f52c0855f3a" xr:uid="{15A93492-DAFA-2845-8CC5-6AA56A81A3CD}"/>
-    <hyperlink ref="A90" r:id="rId18" display="https://scs-ontouml.eemcs.utwente.nl/model/06130cd9-ba26-4324-9f1e-88bd03b88ca9" xr:uid="{C8F0AAC8-E15C-1C40-84AD-77046731CC14}"/>
-    <hyperlink ref="A52" r:id="rId19" display="https://earthportal.eu/ontologies/NVS_P07" xr:uid="{736D9821-6418-B042-A265-9F93FEBFC2AB}"/>
-    <hyperlink ref="B20" r:id="rId20" display="https://ontobee.org/ontology/CHMO" xr:uid="{D80FD32C-0186-074E-A789-BA63C3C0FBA2}"/>
-    <hyperlink ref="C90" r:id="rId21" xr:uid="{FA229F1B-6A23-4D4F-9F4B-A36373D74F93}"/>
-    <hyperlink ref="C17" r:id="rId22" xr:uid="{C2E8234F-2FE4-6F42-B474-076224A40CF9}"/>
-    <hyperlink ref="C77" r:id="rId23" xr:uid="{9D2AB138-A508-0C43-BF5D-6A7912111510}"/>
-    <hyperlink ref="C25" r:id="rId24" xr:uid="{B570D235-B996-7644-80AC-4CD5B56BE905}"/>
-    <hyperlink ref="C46" r:id="rId25" location="IntegrationTime" xr:uid="{5959054A-F7E7-8542-8583-0A4558203518}"/>
-    <hyperlink ref="C48" r:id="rId26" location="IntegrationTime" xr:uid="{1A64D5B5-27D6-CF42-BC35-2479D2C36AED}"/>
-    <hyperlink ref="C2" r:id="rId27" xr:uid="{555FFEC9-5DBF-7E47-A4C5-DF9FC5B70EEF}"/>
-    <hyperlink ref="C30" r:id="rId28" xr:uid="{8104D6FC-1ECF-DC4C-8655-94D174EC37CC}"/>
-    <hyperlink ref="C63" r:id="rId29" xr:uid="{1C9B4C0D-6549-CD44-B478-E27B648E157F}"/>
-    <hyperlink ref="C24" r:id="rId30" xr:uid="{A852BE4A-D08B-6946-B29D-45CBCF0394DD}"/>
-    <hyperlink ref="C67" r:id="rId31" xr:uid="{3B72C5B5-48F0-1E46-A319-25228DF071D2}"/>
-    <hyperlink ref="C68" r:id="rId32" xr:uid="{AB328289-A6B1-A24B-8D21-A5BEBDD8F017}"/>
-    <hyperlink ref="C69" r:id="rId33" xr:uid="{F2496C0E-1F74-1443-B9AA-12A2AA4BD022}"/>
-    <hyperlink ref="C51" r:id="rId34" xr:uid="{1A706F58-35D7-0542-8C3B-2D83812A6BC4}"/>
-    <hyperlink ref="C65" r:id="rId35" xr:uid="{634BD972-B958-864D-A34A-ED64E1A54F14}"/>
-    <hyperlink ref="C62" r:id="rId36" xr:uid="{40641FB9-AD2F-1A47-8768-874BF77204F6}"/>
-    <hyperlink ref="C89" r:id="rId37" xr:uid="{E0E26C66-761F-854D-979B-011E460B7BB4}"/>
-    <hyperlink ref="C60" r:id="rId38" xr:uid="{BEF1E317-B39A-4C41-A822-29A9E0AECDC6}"/>
-    <hyperlink ref="C76" r:id="rId39" xr:uid="{FFDDE5B3-5EE4-1749-9283-B2404C450D47}"/>
-    <hyperlink ref="C88" r:id="rId40" xr:uid="{DBB12542-F692-2D44-8CC1-2B25F55AAD71}"/>
-    <hyperlink ref="C56" r:id="rId41" xr:uid="{5987C402-1AD0-6D41-A7D9-03F070A22118}"/>
-    <hyperlink ref="C55" r:id="rId42" xr:uid="{150DE845-C329-BE4C-8356-8A23832BDA6C}"/>
-    <hyperlink ref="C32" r:id="rId43" xr:uid="{42A2ED53-4748-F144-8042-83EA3FAEFFA5}"/>
-    <hyperlink ref="C87" r:id="rId44" xr:uid="{34A568F4-314D-DC45-9FCD-09BA8D852696}"/>
-    <hyperlink ref="C86" r:id="rId45" xr:uid="{6B71E233-8757-2F44-9B59-3AC56BC52D0C}"/>
-    <hyperlink ref="C57" r:id="rId46" xr:uid="{16A8DEC0-BB7C-9E4A-98B5-FCE7FCC17235}"/>
-    <hyperlink ref="C58" r:id="rId47" xr:uid="{05EB2E2A-9E63-E44D-A471-922CC35999FF}"/>
-    <hyperlink ref="C85" r:id="rId48" xr:uid="{37DA00E0-DBDE-954F-8690-A8F468128B22}"/>
-    <hyperlink ref="C50" r:id="rId49" xr:uid="{39E38128-6CD3-4F43-9AC7-CF7D9BE6C2A7}"/>
-    <hyperlink ref="C49" r:id="rId50" xr:uid="{CC63136F-DDDE-0E4A-9C74-5CF0B3DA4AE0}"/>
-    <hyperlink ref="C42" r:id="rId51" xr:uid="{D64E825D-1515-7747-B40D-8BB67687D95E}"/>
-    <hyperlink ref="C41" r:id="rId52" xr:uid="{FC234C3F-958C-5D40-B086-278A90BA0EF1}"/>
-    <hyperlink ref="C31" r:id="rId53" xr:uid="{695DC735-428C-B641-B857-BE4BABD039B4}"/>
-    <hyperlink ref="C33" r:id="rId54" xr:uid="{A6123D3B-9344-4648-A798-C9656105EC8E}"/>
-    <hyperlink ref="C27" r:id="rId55" xr:uid="{FAC8521C-4FCA-F948-A085-6440C8E00231}"/>
-    <hyperlink ref="C37" r:id="rId56" xr:uid="{D38C8FF9-E399-C041-A2E3-AFB79B4566B1}"/>
-    <hyperlink ref="C36" r:id="rId57" xr:uid="{F63B92C4-2FC2-4D43-8C6F-9C661D780DD5}"/>
-    <hyperlink ref="C35" r:id="rId58" xr:uid="{A571D68F-535D-D14F-8880-19F19B69EEE5}"/>
-    <hyperlink ref="C26" r:id="rId59" xr:uid="{C22900F2-9599-4B45-A290-FB71BBD4FF5B}"/>
-    <hyperlink ref="C29" r:id="rId60" xr:uid="{8223A1A7-D0DE-AA4B-B603-47062E37F784}"/>
-    <hyperlink ref="C74" r:id="rId61" xr:uid="{491775E5-F6D6-3C4D-BA3E-FDF22E9AB107}"/>
-    <hyperlink ref="C73" r:id="rId62" xr:uid="{F6DAB0F7-E03C-6244-A128-6CA285F0E2A4}"/>
-    <hyperlink ref="C72" r:id="rId63" xr:uid="{17948612-13E1-F149-93B9-52D5F110C470}"/>
-    <hyperlink ref="C71" r:id="rId64" xr:uid="{E4A8AFB7-C66A-3240-BF7D-F2916C093943}"/>
-    <hyperlink ref="C82" r:id="rId65" xr:uid="{C497F7E2-44E7-6E4C-9415-4899C4175F6C}"/>
-    <hyperlink ref="C21" r:id="rId66" xr:uid="{7BC2260B-5940-E74A-A602-B4B86FC797AF}"/>
-    <hyperlink ref="C22" r:id="rId67" xr:uid="{9C45F978-C4FF-5048-930F-BE11F56D1C53}"/>
-    <hyperlink ref="C20" r:id="rId68" xr:uid="{80DD7C05-67E3-0740-BF49-6E58E3E96F3C}"/>
-    <hyperlink ref="C18" r:id="rId69" xr:uid="{1AC78E80-6D26-9741-B8D8-341DC6142958}"/>
-    <hyperlink ref="C12" r:id="rId70" xr:uid="{87AABB3A-A36D-5A42-9490-9C02BDBF3ACA}"/>
-    <hyperlink ref="C10" r:id="rId71" xr:uid="{EE9AD4F8-3C82-DB49-B3CF-9DEC32F45D34}"/>
-    <hyperlink ref="C8" r:id="rId72" xr:uid="{10AD49BC-9BE8-D049-95CD-2C518E2353F0}"/>
-    <hyperlink ref="C13" r:id="rId73" xr:uid="{4370A7CB-AB57-B84F-9241-5D6324A48F1A}"/>
-    <hyperlink ref="C75" r:id="rId74" xr:uid="{A5AA1886-54E0-5149-AE81-CBA997AA90AF}"/>
-    <hyperlink ref="C3" r:id="rId75" xr:uid="{A0E7AA6A-89DB-EC4B-8836-4EC86341F9DD}"/>
-    <hyperlink ref="C7" r:id="rId76" xr:uid="{32CD64DA-7FE0-7B40-A2C5-15EC589F8D17}"/>
-    <hyperlink ref="C4" r:id="rId77" xr:uid="{6CF857B4-8FB8-114F-8A69-4AD1B1F35974}"/>
-    <hyperlink ref="C9" r:id="rId78" xr:uid="{7136ECA6-283D-874C-B90C-8E7F28251500}"/>
-    <hyperlink ref="C39" r:id="rId79" xr:uid="{5D63D260-C4DB-6F4A-ADEC-AF6FBC11A7DD}"/>
-    <hyperlink ref="C91" r:id="rId80" xr:uid="{EAA5189B-F422-1246-8B84-C62DB7CF2462}"/>
+    <hyperlink ref="C90" r:id="rId8" xr:uid="{FA229F1B-6A23-4D4F-9F4B-A36373D74F93}"/>
+    <hyperlink ref="C17" r:id="rId9" xr:uid="{C2E8234F-2FE4-6F42-B474-076224A40CF9}"/>
+    <hyperlink ref="C77" r:id="rId10" xr:uid="{9D2AB138-A508-0C43-BF5D-6A7912111510}"/>
+    <hyperlink ref="C25" r:id="rId11" xr:uid="{B570D235-B996-7644-80AC-4CD5B56BE905}"/>
+    <hyperlink ref="C46" r:id="rId12" location="IntegrationTime" xr:uid="{5959054A-F7E7-8542-8583-0A4558203518}"/>
+    <hyperlink ref="C48" r:id="rId13" location="IntegrationTime" xr:uid="{1A64D5B5-27D6-CF42-BC35-2479D2C36AED}"/>
+    <hyperlink ref="C2" r:id="rId14" xr:uid="{555FFEC9-5DBF-7E47-A4C5-DF9FC5B70EEF}"/>
+    <hyperlink ref="C30" r:id="rId15" xr:uid="{8104D6FC-1ECF-DC4C-8655-94D174EC37CC}"/>
+    <hyperlink ref="C63" r:id="rId16" xr:uid="{1C9B4C0D-6549-CD44-B478-E27B648E157F}"/>
+    <hyperlink ref="C24" r:id="rId17" xr:uid="{A852BE4A-D08B-6946-B29D-45CBCF0394DD}"/>
+    <hyperlink ref="C67" r:id="rId18" xr:uid="{3B72C5B5-48F0-1E46-A319-25228DF071D2}"/>
+    <hyperlink ref="C68" r:id="rId19" xr:uid="{AB328289-A6B1-A24B-8D21-A5BEBDD8F017}"/>
+    <hyperlink ref="C69" r:id="rId20" xr:uid="{F2496C0E-1F74-1443-B9AA-12A2AA4BD022}"/>
+    <hyperlink ref="C51" r:id="rId21" xr:uid="{1A706F58-35D7-0542-8C3B-2D83812A6BC4}"/>
+    <hyperlink ref="C65" r:id="rId22" xr:uid="{634BD972-B958-864D-A34A-ED64E1A54F14}"/>
+    <hyperlink ref="C62" r:id="rId23" xr:uid="{40641FB9-AD2F-1A47-8768-874BF77204F6}"/>
+    <hyperlink ref="C89" r:id="rId24" xr:uid="{E0E26C66-761F-854D-979B-011E460B7BB4}"/>
+    <hyperlink ref="C60" r:id="rId25" xr:uid="{BEF1E317-B39A-4C41-A822-29A9E0AECDC6}"/>
+    <hyperlink ref="C76" r:id="rId26" xr:uid="{FFDDE5B3-5EE4-1749-9283-B2404C450D47}"/>
+    <hyperlink ref="C88" r:id="rId27" xr:uid="{DBB12542-F692-2D44-8CC1-2B25F55AAD71}"/>
+    <hyperlink ref="C56" r:id="rId28" xr:uid="{5987C402-1AD0-6D41-A7D9-03F070A22118}"/>
+    <hyperlink ref="C55" r:id="rId29" xr:uid="{150DE845-C329-BE4C-8356-8A23832BDA6C}"/>
+    <hyperlink ref="C32" r:id="rId30" xr:uid="{42A2ED53-4748-F144-8042-83EA3FAEFFA5}"/>
+    <hyperlink ref="C87" r:id="rId31" xr:uid="{34A568F4-314D-DC45-9FCD-09BA8D852696}"/>
+    <hyperlink ref="C86" r:id="rId32" xr:uid="{6B71E233-8757-2F44-9B59-3AC56BC52D0C}"/>
+    <hyperlink ref="C57" r:id="rId33" xr:uid="{16A8DEC0-BB7C-9E4A-98B5-FCE7FCC17235}"/>
+    <hyperlink ref="C58" r:id="rId34" xr:uid="{05EB2E2A-9E63-E44D-A471-922CC35999FF}"/>
+    <hyperlink ref="C85" r:id="rId35" xr:uid="{37DA00E0-DBDE-954F-8690-A8F468128B22}"/>
+    <hyperlink ref="C50" r:id="rId36" xr:uid="{39E38128-6CD3-4F43-9AC7-CF7D9BE6C2A7}"/>
+    <hyperlink ref="C49" r:id="rId37" xr:uid="{CC63136F-DDDE-0E4A-9C74-5CF0B3DA4AE0}"/>
+    <hyperlink ref="C42" r:id="rId38" xr:uid="{D64E825D-1515-7747-B40D-8BB67687D95E}"/>
+    <hyperlink ref="C41" r:id="rId39" xr:uid="{FC234C3F-958C-5D40-B086-278A90BA0EF1}"/>
+    <hyperlink ref="C33" r:id="rId40" xr:uid="{A6123D3B-9344-4648-A798-C9656105EC8E}"/>
+    <hyperlink ref="C27" r:id="rId41" xr:uid="{FAC8521C-4FCA-F948-A085-6440C8E00231}"/>
+    <hyperlink ref="C37" r:id="rId42" xr:uid="{D38C8FF9-E399-C041-A2E3-AFB79B4566B1}"/>
+    <hyperlink ref="C36" r:id="rId43" xr:uid="{F63B92C4-2FC2-4D43-8C6F-9C661D780DD5}"/>
+    <hyperlink ref="C35" r:id="rId44" xr:uid="{A571D68F-535D-D14F-8880-19F19B69EEE5}"/>
+    <hyperlink ref="C26" r:id="rId45" xr:uid="{C22900F2-9599-4B45-A290-FB71BBD4FF5B}"/>
+    <hyperlink ref="C29" r:id="rId46" xr:uid="{8223A1A7-D0DE-AA4B-B603-47062E37F784}"/>
+    <hyperlink ref="C74" r:id="rId47" xr:uid="{491775E5-F6D6-3C4D-BA3E-FDF22E9AB107}"/>
+    <hyperlink ref="C73" r:id="rId48" xr:uid="{F6DAB0F7-E03C-6244-A128-6CA285F0E2A4}"/>
+    <hyperlink ref="C72" r:id="rId49" xr:uid="{17948612-13E1-F149-93B9-52D5F110C470}"/>
+    <hyperlink ref="C71" r:id="rId50" xr:uid="{E4A8AFB7-C66A-3240-BF7D-F2916C093943}"/>
+    <hyperlink ref="C82" r:id="rId51" xr:uid="{C497F7E2-44E7-6E4C-9415-4899C4175F6C}"/>
+    <hyperlink ref="C21" r:id="rId52" xr:uid="{7BC2260B-5940-E74A-A602-B4B86FC797AF}"/>
+    <hyperlink ref="C22" r:id="rId53" xr:uid="{9C45F978-C4FF-5048-930F-BE11F56D1C53}"/>
+    <hyperlink ref="C20" r:id="rId54" xr:uid="{80DD7C05-67E3-0740-BF49-6E58E3E96F3C}"/>
+    <hyperlink ref="C18" r:id="rId55" xr:uid="{1AC78E80-6D26-9741-B8D8-341DC6142958}"/>
+    <hyperlink ref="C12" r:id="rId56" xr:uid="{87AABB3A-A36D-5A42-9490-9C02BDBF3ACA}"/>
+    <hyperlink ref="C10" r:id="rId57" xr:uid="{EE9AD4F8-3C82-DB49-B3CF-9DEC32F45D34}"/>
+    <hyperlink ref="C8" r:id="rId58" xr:uid="{10AD49BC-9BE8-D049-95CD-2C518E2353F0}"/>
+    <hyperlink ref="C13" r:id="rId59" xr:uid="{4370A7CB-AB57-B84F-9241-5D6324A48F1A}"/>
+    <hyperlink ref="C75" r:id="rId60" xr:uid="{A5AA1886-54E0-5149-AE81-CBA997AA90AF}"/>
+    <hyperlink ref="C3" r:id="rId61" xr:uid="{A0E7AA6A-89DB-EC4B-8836-4EC86341F9DD}"/>
+    <hyperlink ref="C7" r:id="rId62" xr:uid="{32CD64DA-7FE0-7B40-A2C5-15EC589F8D17}"/>
+    <hyperlink ref="C4" r:id="rId63" xr:uid="{6CF857B4-8FB8-114F-8A69-4AD1B1F35974}"/>
+    <hyperlink ref="C9" r:id="rId64" xr:uid="{7136ECA6-283D-874C-B90C-8E7F28251500}"/>
+    <hyperlink ref="C39" r:id="rId65" xr:uid="{5D63D260-C4DB-6F4A-ADEC-AF6FBC11A7DD}"/>
+    <hyperlink ref="C91" r:id="rId66" xr:uid="{EAA5189B-F422-1246-8B84-C62DB7CF2462}"/>
+    <hyperlink ref="C92" r:id="rId67" xr:uid="{9507EB4B-76A4-9540-A092-F67FD17BEB72}"/>
+    <hyperlink ref="C95" r:id="rId68" xr:uid="{5D532F7B-1C61-CC4D-9505-805B3D63EEE2}"/>
+    <hyperlink ref="C98" r:id="rId69" xr:uid="{0C3A6049-5147-7A45-BCA9-2534AFBF7606}"/>
+    <hyperlink ref="C99" r:id="rId70" xr:uid="{F5C1E803-01B9-4143-A9A1-0387C2503AA7}"/>
+    <hyperlink ref="C100" r:id="rId71" xr:uid="{D545A560-0AEE-C14A-9898-79DE08027220}"/>
+    <hyperlink ref="C23" r:id="rId72" xr:uid="{3DCBE2A2-2E30-D940-B1C7-50217197C749}"/>
+    <hyperlink ref="C101" r:id="rId73" xr:uid="{8EE434DE-6C31-8A42-AFD0-ACF96FACD731}"/>
+    <hyperlink ref="C31" r:id="rId74" xr:uid="{695DC735-428C-B641-B857-BE4BABD039B4}"/>
+    <hyperlink ref="C102" r:id="rId75" xr:uid="{3C7B66EE-7201-C941-91F2-8482A69E6644}"/>
+    <hyperlink ref="C96" r:id="rId76" xr:uid="{0088B82E-D5C1-304B-A607-2B94402A5B5B}"/>
+    <hyperlink ref="C93" r:id="rId77" xr:uid="{3B42A478-992F-E24B-AC69-38F9B0C838A2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -3080,7 +3321,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE73302C-2B5F-6D41-A45E-E19459CB0D2B}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -3090,83 +3331,88 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>297</v>
+        <v>290</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>